<commit_message>
rad: dnevni zapis 2026-09-06 (automatski, scripts/rad-dnevno.ps1)
</commit_message>
<xml_diff>
--- a/docs/records/RAD.xlsx
+++ b/docs/records/RAD.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upute" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Isporuke'!$A$1:$E$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Isporuke'!$A$1:$E$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Vizije'!$A$1:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -228,12 +228,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$12</f>
+              <f>'Sažetak'!$A$6:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$6:$B$12</f>
+              <f>'Sažetak'!$B$6:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -317,12 +317,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$12</f>
+              <f>'Sažetak'!$A$6:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$C$6:$C$12</f>
+              <f>'Sažetak'!$C$6:$C$13</f>
             </numRef>
           </val>
         </ser>
@@ -398,12 +398,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$12</f>
+              <f>'Sažetak'!$A$6:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$D$6:$D$12</f>
+              <f>'Sažetak'!$D$6:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -480,12 +480,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$12</f>
+              <f>'Sažetak'!$A$6:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$E$6:$E$12</f>
+              <f>'Sažetak'!$E$6:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -551,7 +551,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B15</f>
+              <f>'Sažetak'!B16</f>
             </strRef>
           </tx>
           <spPr>
@@ -561,12 +561,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$16:$A$20</f>
+              <f>'Sažetak'!$A$17:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$16:$B$20</f>
+              <f>'Sažetak'!$B$17:$B$21</f>
             </numRef>
           </val>
         </ser>
@@ -612,7 +612,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!D15</f>
+              <f>'Sažetak'!D16</f>
             </strRef>
           </tx>
           <spPr>
@@ -622,12 +622,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$16:$A$20</f>
+              <f>'Sažetak'!$A$17:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$D$16:$D$20</f>
+              <f>'Sažetak'!$D$17:$D$21</f>
             </numRef>
           </val>
         </ser>
@@ -694,7 +694,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B44</f>
+              <f>'Sažetak'!B45</f>
             </strRef>
           </tx>
           <spPr>
@@ -704,12 +704,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$45:$A$55</f>
+              <f>'Sažetak'!$A$46:$A$56</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$45:$B$55</f>
+              <f>'Sažetak'!$B$46:$B$56</f>
             </numRef>
           </val>
         </ser>
@@ -718,7 +718,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!C44</f>
+              <f>'Sažetak'!C45</f>
             </strRef>
           </tx>
           <spPr>
@@ -728,12 +728,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$45:$A$55</f>
+              <f>'Sažetak'!$A$46:$A$56</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$C$45:$C$55</f>
+              <f>'Sažetak'!$C$46:$C$56</f>
             </numRef>
           </val>
         </ser>
@@ -801,7 +801,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B58</f>
+              <f>'Sažetak'!B59</f>
             </strRef>
           </tx>
           <spPr>
@@ -811,12 +811,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$59:$A$64</f>
+              <f>'Sažetak'!$A$60:$A$65</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$59:$B$64</f>
+              <f>'Sažetak'!$B$60:$B$65</f>
             </numRef>
           </val>
         </ser>
@@ -1326,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1349,7 +1349,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generirano 2026-09-05 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
+          <t>Generirano 2026-09-06 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
         </is>
       </c>
     </row>
@@ -1577,13 +1577,13 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6902</v>
+        <v>6978</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>11.6</v>
@@ -1598,162 +1598,175 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>139</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1993</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>VRSTE RADA (po commitima; „ručno" pregazi „auto")</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>vrsta rada</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>commita</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>udio</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>redaka (+/−)</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>planiranje</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>2982</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>vođenje dokumentacije</t>
+          <t>planiranje</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.285</v>
+        <v>0.122</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>1811</v>
+        <v>3027</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>izvođenje procesa</t>
+          <t>vođenje dokumentacije</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.333</v>
+        <v>0.324</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>18162</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>poliranje koda</t>
+          <t>izvođenje procesa</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.187</v>
+        <v>0.331</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>26569</v>
+        <v>20064</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>poliranje koda</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>26569</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>debugging</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="D20" s="5" t="n">
+      <c r="C21" s="6" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="D21" s="5" t="n">
         <v>3333</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>KVALITETA I BRZINA (razdoblje od 2026-08-29)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>pokazatelj</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>vrijednost</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>što je to</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>radnih dana (dana s commitom)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>commita</t>
+          <t>radnih dana (dana s commitom)</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>123</v>
+        <v>8</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
@@ -1764,11 +1777,11 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>commita po radnom danu</t>
+          <t>commita</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>17.6</v>
+        <v>139</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -1779,11 +1792,11 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>isporuka (PROGRESS unosa)</t>
+          <t>commita po radnom danu</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>89</v>
+        <v>17.4</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -1794,11 +1807,11 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>isporuka po radnom danu</t>
+          <t>isporuka (PROGRESS unosa)</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>12.7</v>
+        <v>95</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -1809,253 +1822,250 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>sati rada (git-hours proxy)</t>
+          <t>isporuka po radnom danu</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>PROXY — razmaci &lt; 2 h među commitima + 0.5 h po sesiji, ne štoperica</t>
+        <v>11.9</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>commita po satu (proxy)</t>
+          <t>sati rada (git-hours proxy)</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>proxy</t>
+        <v>66.90000000000001</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>PROXY — razmaci &lt; 2 h među commitima + 0.5 h po sesiji, ne štoperica</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>redaka promijenjeno (+/−)</t>
+          <t>commita po satu (proxy)</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>52857</v>
+        <v>2.1</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>mjera</t>
+          <t>proxy</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>redaka u testovima i branama</t>
+          <t>redaka promijenjeno (+/−)</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>5280</v>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko rada ide u dokaz, ne u tvrdnju</t>
+        <v>54926</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>udio testnih redaka</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+          <t>redaka u testovima i branama</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6068</v>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>mjera — koliko rada ide u dokaz, ne u tvrdnju</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>deploya na produkciju</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>7</v>
+          <t>udio testnih redaka</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>0.11</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>mjera (🚀 u PROGRESS.md)</t>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>debugging commita</t>
+          <t>deploya na produkciju</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko se vraćamo na već napravljeno</t>
+        <v>7</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>mjera (🚀 u PROGRESS.md)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>udio debugginga</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n">
-        <v>0.065</v>
+          <t>debugging commita</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>niže = bolje, ali 0 znači da brane ne rade</t>
+          <t>mjera — koliko se vraćamo na već napravljeno</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>udio dokumentacije</t>
+          <t>udio debugginga</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.285</v>
+        <v>0.058</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>režija: pravilo #3 + #6 (audit prije compacta)</t>
+          <t>niže = bolje, ali 0 znači da brane ne rade</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>CI-padova popravljenih</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+          <t>udio dokumentacije</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>režija: pravilo #3 + #6 (audit prije compacta)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>isporuka pokrenutih Leonovim nalazom</t>
+          <t>CI-padova popravljenih</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko smjera dolazi s uređaja, ne iz plana</t>
+        <v>2</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>zatvorenih faza u razdoblju</t>
+          <t>isporuka pokrenutih Leonovim nalazom</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+        <v>18</v>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>mjera — koliko smjera dolazi s uređaja, ne iz plana</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
+          <t>zatvorenih faza u razdoblju</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>prosječno trajanje zatvorene faze (dana)</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B42" s="5" t="n">
         <v>8.5</v>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>mjera — sve zatvorene faze na listu Faze</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>FAZE — gotovo / preostalo (cigle)</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>faza</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>gotove cigle</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>preostale cigle</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>stanje</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Osobni UGC-graditelj F1–F5</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>zatvoreno</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Frontend redizajn C0–C7 + KOSTUR·TELEFON</t>
+          <t>Osobni UGC-graditelj F1–F5</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="C46" s="5" t="n">
         <v>0</v>
@@ -2069,11 +2079,11 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>MREŽA — sanacija A–E</t>
+          <t>Frontend redizajn C0–C7 + KOSTUR·TELEFON</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="C47" s="5" t="n">
         <v>0</v>
@@ -2087,11 +2097,11 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>RAČUN R1 — OAuth + upitnik + dijalog</t>
+          <t>MREŽA — sanacija A–E</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C48" s="5" t="n">
         <v>0</v>
@@ -2105,50 +2115,50 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>F1 · UREĐAJ</t>
+          <t>RAČUN R1 — OAuth + upitnik + dijalog</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>u tijeku</t>
+          <t>zatvoreno</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>F2 · RAČUN</t>
+          <t>F1 · UREĐAJ</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C50" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>planirano</t>
+          <t>u tijeku</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>F3 · DVOJEZIČNOST</t>
+          <t>F2 · RAČUN</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
@@ -2159,14 +2169,14 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>F4 · ČIŠĆENJE</t>
+          <t>F3 · DVOJEZIČNOST</t>
         </is>
       </c>
       <c r="B52" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
@@ -2177,14 +2187,14 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>F5 · VJEŽBE</t>
+          <t>F4 · ČIŠĆENJE</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
@@ -2195,7 +2205,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>F6 · MCP</t>
+          <t>F5 · VJEŽBE</t>
         </is>
       </c>
       <c r="B54" s="5" t="n">
@@ -2213,7 +2223,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>F7 · OBJAVA</t>
+          <t>F6 · MCP</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
@@ -2228,39 +2238,47 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>F7 · OBJAVA</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>planirano</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>PLANOVI I VIZIJE — po stanju</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>stanje</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>stavki</t>
         </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>isporučeno</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>planirano</t>
+          <t>isporučeno</t>
         </is>
       </c>
       <c r="B60" s="5" t="n">
@@ -2270,40 +2288,50 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>pokrenuto</t>
+          <t>planirano</t>
         </is>
       </c>
       <c r="B61" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>ideja</t>
+          <t>pokrenuto</t>
         </is>
       </c>
       <c r="B62" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>parkirano</t>
+          <t>ideja</t>
         </is>
       </c>
       <c r="B63" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
+          <t>parkirano</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
           <t>odbijeno</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n">
+      <c r="B65" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2319,7 +2347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8312,8 +8340,756 @@
         <v>0</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>23:57</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>cbaf4d2</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t>rad: dnevni zapis 2026-09-05 (automatski, scripts/rad-dnevno.ps1)</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr"/>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr"/>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I125" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J125" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K125" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>23:58</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>26e4965</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t>rad: RAD.xlsx se puni AUTOMATSKI svaki dan 23:45 -- scripts/rad-dnevno.ps1 + Windows Task Scheduler (Leon: "to treba biti automatski")</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr"/>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr"/>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I126" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J126" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="K126" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L126" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>00:50</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>93b4897</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>docs: Leonov odgovor §6/1 -- odjava brise lokalni izbor teme (F2/1); iPhone-nalaz o stipanju opisuje PRODUKCIJU (instalirana app), ne F1/11</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr"/>
+      <c r="H127" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I127" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="K127" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="L127" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>01:48</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>4d8f19b</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t>F1/4: popis tema ima JEDNO mjesto -- scripts/teme.js cita tokens.css za sve cetiri brane; a11y-brana prvi put skenira carbon</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>F1/4</t>
+        </is>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G128" s="5" t="inlineStr"/>
+      <c r="H128" s="5" t="inlineStr">
+        <is>
+          <t>brane i mjerenje</t>
+        </is>
+      </c>
+      <c r="I128" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="J128" s="5" t="n">
+        <v>193</v>
+      </c>
+      <c r="K128" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="L128" s="5" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>01:54</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>0785952</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t>F1/5: pravne stranice prate uredjaj -- boot.js (sinkron) + data-theme na contact/faq/privacy/terms; legal.spec mjeri iscrtano dark→carbon / light→academic</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>F1/5</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr"/>
+      <c r="H129" s="5" t="inlineStr">
+        <is>
+          <t>cigla</t>
+        </is>
+      </c>
+      <c r="I129" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J129" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="K129" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="L129" s="5" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>02:09</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>2d45182</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>docs: Leonove stavke 06.09. SAMO ZAPISANE -- FAQ/About/kontakt sokrat@sokratstudy.com (F3/1 dopuna, prije prijevoda) · "uvijek bijela" = produkcija bez F1/5 · "Automatic · Carbon" u biracu = pitanje §6/7</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr"/>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr"/>
+      <c r="H130" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I130" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J130" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="K130" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L130" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>02:38</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>a354960</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>docs/compact-prep: HISTORY dobiva redak 2026-09-06 (F1/4 + F1/5 bili zalijepljeni na 05.09.) · CLAUDE.md: F1 gotov osim F1/9</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr"/>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr"/>
+      <c r="H131" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I131" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J131" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K131" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L131" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>02:38</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>4cce27b</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="inlineStr">
+        <is>
+          <t>docs: CLAUDE.md natrag pod budzet -- dva retka stanja F1 sazeta u jedan (prethodni commit je prosao jer je `| tail` progutao pad check:docs)</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr"/>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr"/>
+      <c r="H132" s="5" t="inlineStr">
+        <is>
+          <t>brane i mjerenje</t>
+        </is>
+      </c>
+      <c r="I132" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J132" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K132" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L132" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>03:28</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>57e2158</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t>F1/9: kartice kao Tinder-spil na dodiru -- palac desno = znam, lijevo = ne znam, spil od tri (samo `pointer: coarse`), strelice kao stolni pandan; jedini put upisa ostaju markKnown/markUnknown</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>F1/9</t>
+        </is>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr"/>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>cigla</t>
+        </is>
+      </c>
+      <c r="I133" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>1201</v>
+      </c>
+      <c r="K133" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="L133" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>03:28</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>d1743a8</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t>docs: HISTORY -- F1 uredjaj: sve cigle isporucene (F1/9 Tinder-spil 57e2158)</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr"/>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr"/>
+      <c r="H134" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I134" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J134" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K134" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L134" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>95e3ba1</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>docs: Tinder-KADAR -- mjerenje (BACKLOG §E) + plan F1/12 kadar · F1/13 listanje (RASPORED) · §6/8 kraj spila; bez koda</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr"/>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>planiranje</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr"/>
+      <c r="H135" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I135" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="K135" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L135" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>04:19</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>182bac3</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t>docs: Leonovi odgovori za Tinder-kadar -- izbornik na kraju spila · ✕ lijevo / strelica desno i na kompu · sve tipkama (X/Z) · F1/14 tutorial (kasnije, ali predvidjen tablicom akcija)</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr"/>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G136" s="5" t="inlineStr"/>
+      <c r="H136" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I136" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J136" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="K136" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L136" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>04:40</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>900f142</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t>docs: anketa -- Leonovih pet odgovora zatvara §6 (sidebar obrisati · vjezbe samo tokeni · Facebook otpao · HR predmeti cekaju F5 recepte · birac samo "Automatski")</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr"/>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr"/>
+      <c r="H137" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K137" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="L137" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>04:55</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>fe1af72</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t>docs: HR autor-bot zapisan kao KASNIJE (Leon 06.09.) -- sto postoji, sto fali, redoslijed kad dodje na red</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr"/>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G138" s="5" t="inlineStr"/>
+      <c r="H138" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I138" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J138" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K138" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>04:58</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>2d07d00</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>docs: HR autor-bot bez API kljuca -- graditelji su Claude Code subagenti, ne Sonnet API (Leon 06.09.)</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr"/>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr"/>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K139" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L139" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>05:03</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>8ec0e18</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t>docs: HR materijali 1. godine postoje na Driveu (Leon 06.09.) -- izvor za autor-bota, jos nepregledano</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr"/>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr"/>
+      <c r="H140" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I140" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J140" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K140" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L140" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L124"/>
+  <autoFilter ref="A1:L140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8324,7 +9100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10408,8 +11184,146 @@
       </c>
       <c r="E90" s="5" t="inlineStr"/>
     </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Leon s previewom F1/9 → Tinder-KADAR (palac lista, gumbi sude, kartica = ekran): IZMJERENO + PLAN, bez koda</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>F1/9: kartice kao Tinder-špil na dodiru (palac · špil · pečati) + strelice kao stolni pandan — F1 uređaj ima sve cigle</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Leonove stavke poslije F1/5, SAMO ZAPISANE (*„Ovo samo zapiši, nemoj ništa raditi"*)</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>F1/5: pravne stranice prate uređaj (`boot.js` sinkron + `data-theme` na 4 stranice) — kraj poliranja F1 osim Tindera</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>F1/4: `scripts/teme.js` — popis tema iz `tokens.css` za sve četiri brane (a11y prvi put skenira `carbon`)</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>FABLE</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Leonovi odgovori: F2/1 = odjava briše lokalni izbor · iPhone: dodir ne zumira, štipanje da — ali testira INSTALIRANU aplikaciju (produkcija, bez F1/11)</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E90"/>
+  <autoFilter ref="A1:E96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10524,22 +11438,22 @@
         <v>5</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
@@ -10709,25 +11623,25 @@
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>8</v>
-      </c>
       <c r="H6" s="5" t="n">
-        <v>0.73</v>
+        <v>0.79</v>
       </c>
       <c r="I6" s="5" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="K6" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>4.5</v>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rad: dnevni zapis 2026-09-07 (automatski, scripts/rad-dnevno.ps1)
</commit_message>
<xml_diff>
--- a/docs/records/RAD.xlsx
+++ b/docs/records/RAD.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upute" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Isporuke'!$A$1:$E$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Isporuke'!$A$1:$E$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Vizije'!$A$1:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -228,12 +228,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$13</f>
+              <f>'Sažetak'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$6:$B$13</f>
+              <f>'Sažetak'!$B$6:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -317,12 +317,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$13</f>
+              <f>'Sažetak'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$C$6:$C$13</f>
+              <f>'Sažetak'!$C$6:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -398,12 +398,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$13</f>
+              <f>'Sažetak'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$D$6:$D$13</f>
+              <f>'Sažetak'!$D$6:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -480,12 +480,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$6:$A$13</f>
+              <f>'Sažetak'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$E$6:$E$13</f>
+              <f>'Sažetak'!$E$6:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -551,7 +551,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B16</f>
+              <f>'Sažetak'!B17</f>
             </strRef>
           </tx>
           <spPr>
@@ -561,12 +561,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$17:$A$21</f>
+              <f>'Sažetak'!$A$18:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$17:$B$21</f>
+              <f>'Sažetak'!$B$18:$B$22</f>
             </numRef>
           </val>
         </ser>
@@ -612,7 +612,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!D16</f>
+              <f>'Sažetak'!D17</f>
             </strRef>
           </tx>
           <spPr>
@@ -622,12 +622,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$17:$A$21</f>
+              <f>'Sažetak'!$A$18:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$D$17:$D$21</f>
+              <f>'Sažetak'!$D$18:$D$22</f>
             </numRef>
           </val>
         </ser>
@@ -694,7 +694,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B45</f>
+              <f>'Sažetak'!B46</f>
             </strRef>
           </tx>
           <spPr>
@@ -704,12 +704,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$46:$A$56</f>
+              <f>'Sažetak'!$A$47:$A$57</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$46:$B$56</f>
+              <f>'Sažetak'!$B$47:$B$57</f>
             </numRef>
           </val>
         </ser>
@@ -718,7 +718,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!C45</f>
+              <f>'Sažetak'!C46</f>
             </strRef>
           </tx>
           <spPr>
@@ -728,12 +728,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$46:$A$56</f>
+              <f>'Sažetak'!$A$47:$A$57</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$C$46:$C$56</f>
+              <f>'Sažetak'!$C$47:$C$57</f>
             </numRef>
           </val>
         </ser>
@@ -801,7 +801,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Sažetak'!B59</f>
+              <f>'Sažetak'!B60</f>
             </strRef>
           </tx>
           <spPr>
@@ -811,12 +811,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Sažetak'!$A$60:$A$65</f>
+              <f>'Sažetak'!$A$61:$A$66</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sažetak'!$B$60:$B$65</f>
+              <f>'Sažetak'!$B$61:$B$66</f>
             </numRef>
           </val>
         </ser>
@@ -1326,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1349,7 +1349,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generirano 2026-09-06 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
+          <t>Generirano 2026-09-07 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
         </is>
       </c>
     </row>
@@ -1605,16 +1605,16 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>1993</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>6</v>
@@ -1626,162 +1626,175 @@
         <v>788</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>1051</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>VRSTE RADA (po commitima; „ručno" pregazi „auto")</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>vrsta rada</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>commita</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>udio</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>redaka (+/−)</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>planiranje</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>3027</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>vođenje dokumentacije</t>
+          <t>planiranje</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.324</v>
+        <v>0.126</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>1933</v>
+        <v>3438</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>izvođenje procesa</t>
+          <t>vođenje dokumentacije</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
         <v>46</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.331</v>
+        <v>0.322</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>20064</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>poliranje koda</t>
+          <t>izvođenje procesa</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0.165</v>
+        <v>0.336</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>26569</v>
+        <v>20640</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>poliranje koda</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>26569</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>debugging</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C21" s="6" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C22" s="6" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="D22" s="5" t="n">
         <v>3333</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>KVALITETA I BRZINA (razdoblje od 2026-08-29)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>pokazatelj</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>vrijednost</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>što je to</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>radnih dana (dana s commitom)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>commita</t>
+          <t>radnih dana (dana s commitom)</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -1792,11 +1805,11 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>commita po radnom danu</t>
+          <t>commita</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>17.4</v>
+        <v>143</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -1807,11 +1820,11 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>isporuka (PROGRESS unosa)</t>
+          <t>commita po radnom danu</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>95</v>
+        <v>15.9</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -1822,11 +1835,11 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>isporuka po radnom danu</t>
+          <t>isporuka (PROGRESS unosa)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>11.9</v>
+        <v>97</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -1837,253 +1850,250 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>sati rada (git-hours proxy)</t>
+          <t>isporuka po radnom danu</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>PROXY — razmaci &lt; 2 h među commitima + 0.5 h po sesiji, ne štoperica</t>
+        <v>10.8</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>commita po satu (proxy)</t>
+          <t>sati rada (git-hours proxy)</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>proxy</t>
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>PROXY — razmaci &lt; 2 h među commitima + 0.5 h po sesiji, ne štoperica</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>redaka promijenjeno (+/−)</t>
+          <t>commita po satu (proxy)</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>54926</v>
+        <v>2</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>mjera</t>
+          <t>proxy</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>redaka u testovima i branama</t>
+          <t>redaka promijenjeno (+/−)</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>6068</v>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko rada ide u dokaz, ne u tvrdnju</t>
+        <v>55977</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>udio testnih redaka</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+          <t>redaka u testovima i branama</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>6288</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>mjera — koliko rada ide u dokaz, ne u tvrdnju</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>deploya na produkciju</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>7</v>
+          <t>udio testnih redaka</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>0.112</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>mjera (🚀 u PROGRESS.md)</t>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>debugging commita</t>
+          <t>deploya na produkciju</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko se vraćamo na već napravljeno</t>
+        <v>7</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>mjera (🚀 u PROGRESS.md)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>udio debugginga</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="n">
-        <v>0.058</v>
+          <t>debugging commita</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>niže = bolje, ali 0 znači da brane ne rade</t>
+          <t>mjera — koliko se vraćamo na već napravljeno</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>udio dokumentacije</t>
+          <t>udio debugginga</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.324</v>
+        <v>0.056</v>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>režija: pravilo #3 + #6 (audit prije compacta)</t>
+          <t>niže = bolje, ali 0 znači da brane ne rade</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>CI-padova popravljenih</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+          <t>udio dokumentacije</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>režija: pravilo #3 + #6 (audit prije compacta)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>isporuka pokrenutih Leonovim nalazom</t>
+          <t>CI-padova popravljenih</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>mjera — koliko smjera dolazi s uređaja, ne iz plana</t>
+        <v>2</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>zatvorenih faza u razdoblju</t>
+          <t>isporuka pokrenutih Leonovim nalazom</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>mjera</t>
+        <v>18</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>mjera — koliko smjera dolazi s uređaja, ne iz plana</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
+          <t>zatvorenih faza u razdoblju</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>mjera</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t>prosječno trajanje zatvorene faze (dana)</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n">
+      <c r="B43" s="5" t="n">
         <v>8.5</v>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>mjera — sve zatvorene faze na listu Faze</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>FAZE — gotovo / preostalo (cigle)</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>faza</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>gotove cigle</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>preostale cigle</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>stanje</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Osobni UGC-graditelj F1–F5</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>zatvoreno</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Frontend redizajn C0–C7 + KOSTUR·TELEFON</t>
+          <t>Osobni UGC-graditelj F1–F5</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="C47" s="5" t="n">
         <v>0</v>
@@ -2097,11 +2107,11 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>MREŽA — sanacija A–E</t>
+          <t>Frontend redizajn C0–C7 + KOSTUR·TELEFON</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="C48" s="5" t="n">
         <v>0</v>
@@ -2115,11 +2125,11 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>RAČUN R1 — OAuth + upitnik + dijalog</t>
+          <t>MREŽA — sanacija A–E</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C49" s="5" t="n">
         <v>0</v>
@@ -2133,50 +2143,50 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>F1 · UREĐAJ</t>
+          <t>RAČUN R1 — OAuth + upitnik + dijalog</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C50" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>u tijeku</t>
+          <t>zatvoreno</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>F2 · RAČUN</t>
+          <t>F1 · UREĐAJ</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>planirano</t>
+          <t>u tijeku</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>F3 · DVOJEZIČNOST</t>
+          <t>F2 · RAČUN</t>
         </is>
       </c>
       <c r="B52" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
@@ -2187,14 +2197,14 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>F4 · ČIŠĆENJE</t>
+          <t>F3 · DVOJEZIČNOST</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
@@ -2205,14 +2215,14 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>F5 · VJEŽBE</t>
+          <t>F4 · ČIŠĆENJE</t>
         </is>
       </c>
       <c r="B54" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
@@ -2223,7 +2233,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>F6 · MCP</t>
+          <t>F5 · VJEŽBE</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
@@ -2241,7 +2251,7 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>F7 · OBJAVA</t>
+          <t>F6 · MCP</t>
         </is>
       </c>
       <c r="B56" s="5" t="n">
@@ -2256,39 +2266,47 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>F7 · OBJAVA</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>planirano</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>PLANOVI I VIZIJE — po stanju</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>stanje</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>stavki</t>
         </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>isporučeno</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>planirano</t>
+          <t>isporučeno</t>
         </is>
       </c>
       <c r="B61" s="5" t="n">
@@ -2298,40 +2316,50 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>pokrenuto</t>
+          <t>planirano</t>
         </is>
       </c>
       <c r="B62" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>ideja</t>
+          <t>pokrenuto</t>
         </is>
       </c>
       <c r="B63" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>parkirano</t>
+          <t>ideja</t>
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
+          <t>parkirano</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
           <t>odbijeno</t>
         </is>
       </c>
-      <c r="B65" s="5" t="n">
+      <c r="B66" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2347,7 +2375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9088,8 +9116,192 @@
         <v>0</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>e6ed07d</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>rad: dnevni zapis 2026-09-06 (automatski, scripts/rad-dnevno.ps1)</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr"/>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr"/>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L141" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>01:16</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>27d495a</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>docs: model monetizacije -- organizacija je najam, firme placaju prve (ADR-036)</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr"/>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>planiranje</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr"/>
+      <c r="H142" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I142" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J142" s="5" t="n">
+        <v>347</v>
+      </c>
+      <c r="K142" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="L142" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>1384f6b</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>docs(progress): sesija 07.09. -- model monetizacije zakljucan, cinjenice o inkubatoru provjerene</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr"/>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>vođenje dokumentacije</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr"/>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="K143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>a341880</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t>Mjerenje aktivacije i povratka: SokratMetrika u consent.js + kuka u switchSection()</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr"/>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr"/>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I144" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J144" s="5" t="n">
+        <v>469</v>
+      </c>
+      <c r="K144" s="5" t="n">
+        <v>107</v>
+      </c>
+      <c r="L144" s="5" t="n">
+        <v>220</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L140"/>
+  <autoFilter ref="A1:L144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9100,7 +9312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11322,8 +11534,54 @@
       </c>
       <c r="E96" s="5" t="inlineStr"/>
     </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>OPUS, DRUGA SESIJA</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Mjerenje aktivacije i povratka isporučeno · gate pristanka obrnuto provjeren</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>OPUS</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Model monetizacije zaključan (ADR-035 + ADR-036) · činjenice o inkubatoru provjerene · KÔD NIJE DIRAN</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>planiranje</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E96"/>
+  <autoFilter ref="A1:E98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11623,7 +11881,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>14</v>
@@ -11635,13 +11893,13 @@
         <v>0.79</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>3.67</v>
+        <v>2.75</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>12</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rad: dnevni zapis 2026-09-08 (automatski, scripts/rad-dnevno.ps1)
</commit_message>
<xml_diff>
--- a/docs/records/RAD.xlsx
+++ b/docs/records/RAD.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upute" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dnevnik'!$A$1:$L$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Isporuke'!$A$1:$E$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Vizije'!$A$1:$E$22</definedName>
   </definedNames>
@@ -1349,7 +1349,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generirano 2026-09-07 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
+          <t>Generirano 2026-09-08 iz gita (od 2026-08-29), PROGRESS.md i RASPORED.md. Pokreni: python scripts/rad-xlsx.py</t>
         </is>
       </c>
     </row>
@@ -1633,16 +1633,16 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>1051</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>2</v>
@@ -1693,7 +1693,7 @@
         <v>18</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.126</v>
+        <v>0.125</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>3438</v>
@@ -1709,7 +1709,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.322</v>
+        <v>0.319</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>1997</v>
@@ -1722,10 +1722,10 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0.336</v>
+        <v>0.34</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>20640</v>
@@ -1741,7 +1741,7 @@
         <v>23</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>0.161</v>
+        <v>0.16</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>26569</v>
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>15.9</v>
+        <v>16</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>69.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.322</v>
+        <v>0.319</v>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
@@ -2375,7 +2375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9300,8 +9300,54 @@
         <v>220</v>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>d5377ff</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>rad: dnevni zapis 2026-09-07 (automatski, scripts/rad-dnevno.ps1)</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr"/>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>izvođenje procesa</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr"/>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>ostalo</t>
+        </is>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L144"/>
+  <autoFilter ref="A1:L145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11881,7 +11927,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>14</v>
@@ -11893,13 +11939,13 @@
         <v>0.79</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>2.75</v>
+        <v>2.2</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>12</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>

</xml_diff>